<commit_message>
feat: เพิ่มคอลัมน์ org_name/position_name ใน import template + fixture
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/import-sample.xlsx
+++ b/backend/tests/fixtures/import-sample.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -427,6 +427,8 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,6 +467,16 @@
           <t>วุฒิ(BACHELOR/MASTER/DOCTORATE)</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>หน่วยงาน</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ตำแหน่ง</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -502,6 +514,16 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>กองบริหารทรัพยากรบุคคล</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>นักทรัพยากรบุคคลชำนาญการ</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -537,6 +559,16 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>MASTER</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>กองบริหารทรัพยากรบุคคล</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ผู้อำนวยการกอง</t>
         </is>
       </c>
     </row>
@@ -697,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -705,6 +737,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -731,6 +764,11 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>ชื่อตำแหน่ง</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>หน่วยงาน</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: HR Import Phase 2 — org/position resolve + upload UI + audit + security (#12)
Phase 2 ของ HR Excel import (ต่อจาก #11):
- 2a backend: find-or-create org/position (เลิก hardcode id=1), History.position_id=NULL, validate required, re-import 1062, parse hardening
- 2b frontend: ImportPage (admin upload UI) + route + sidebar + single-source template
- 2c: JWT alg HS256-only, import endpoint robustness (rate limit/magic bytes/size/audit)
- migrations: import_log (audit) + UNIQUE SHA2 generated column + FK indexes (TiDB-safe) + FK users
- PR-0: SSL CA fail-closed
- CI/deploy workflows disabled (Actions quota); verify ผ่าน local Docker 59/100 OK
Deploy: ดู docs/deploy-hr-import-phase2.md (ตั้ง MYSQL_SSL_CA + apply migration บน TiDB ก่อน import)
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/import-sample.xlsx
+++ b/backend/tests/fixtures/import-sample.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -427,6 +427,8 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,6 +467,16 @@
           <t>วุฒิ(BACHELOR/MASTER/DOCTORATE)</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>หน่วยงาน</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ตำแหน่ง</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -502,6 +514,16 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>กองบริหารทรัพยากรบุคคล</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>นักทรัพยากรบุคคลชำนาญการ</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -537,6 +559,16 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>MASTER</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>กองบริหารทรัพยากรบุคคล</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ผู้อำนวยการกอง</t>
         </is>
       </c>
     </row>
@@ -697,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -705,6 +737,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -731,6 +764,11 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>ชื่อตำแหน่ง</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>หน่วยงาน</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: require Thai citizen ID checksum on new personnel writes
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/import-sample.xlsx
+++ b/backend/tests/fixtures/import-sample.xlsx
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>1100100299001</t>
+          <t>1100100299005</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1100100299002</t>
+          <t>1100100299013</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>1100100299001</t>
+          <t>1100100299005</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>